<commit_message>
rerun so the reports, workbooks and figures carry the shorter text
</commit_message>
<xml_diff>
--- a/01_Preprocess/01_Filtering/c_data/01_filter.xlsx
+++ b/01_Preprocess/01_Filtering/c_data/01_filter.xlsx
@@ -392,7 +392,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Precursors, protein groups and share of starting signal after each filter</t>
+          <t>Rows, groups and signal after each filter</t>
         </is>
       </c>
     </row>
@@ -410,7 +410,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Contaminant symbol strings removed, how each matched, and the signal it carried</t>
+          <t>Removed contaminants and their signal</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rerun reports, workbooks and figures with shorter text
</commit_message>
<xml_diff>
--- a/01_Preprocess/01_Filtering/c_data/01_filter.xlsx
+++ b/01_Preprocess/01_Filtering/c_data/01_filter.xlsx
@@ -392,7 +392,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Precursors, protein groups and share of starting signal after each filter</t>
+          <t>Rows, groups and signal after each filter</t>
         </is>
       </c>
     </row>
@@ -410,7 +410,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Contaminant symbol strings removed, how each matched, and the signal it carried</t>
+          <t>Removed contaminants and their signal</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rerun all stages on repaired precursors and update quoted numbers
</commit_message>
<xml_diff>
--- a/01_Preprocess/01_Filtering/c_data/01_filter.xlsx
+++ b/01_Preprocess/01_Filtering/c_data/01_filter.xlsx
@@ -5941,13 +5941,13 @@
         </is>
       </c>
       <c r="B2">
-        <v>53760</v>
+        <v>53744</v>
       </c>
       <c r="C2">
-        <v>3736</v>
+        <v>3734</v>
       </c>
       <c r="D2">
-        <v>99.72765070997796</v>
+        <v>98.58844075613163</v>
       </c>
     </row>
     <row r="3">
@@ -5957,13 +5957,13 @@
         </is>
       </c>
       <c r="B3">
-        <v>49801</v>
+        <v>49871</v>
       </c>
       <c r="C3">
         <v>3664</v>
       </c>
       <c r="D3">
-        <v>85.94764178778486</v>
+        <v>87.63098062339989</v>
       </c>
     </row>
     <row r="4">
@@ -5973,13 +5973,13 @@
         </is>
       </c>
       <c r="B4">
-        <v>49788</v>
+        <v>49858</v>
       </c>
       <c r="C4">
         <v>3662</v>
       </c>
       <c r="D4">
-        <v>85.94736147006761</v>
+        <v>87.63070030568271</v>
       </c>
     </row>
     <row r="5">
@@ -5989,13 +5989,13 @@
         </is>
       </c>
       <c r="B5">
-        <v>47133</v>
+        <v>47201</v>
       </c>
       <c r="C5">
         <v>3451</v>
       </c>
       <c r="D5">
-        <v>57.99577454956071</v>
+        <v>59.67866240498889</v>
       </c>
     </row>
   </sheetData>
@@ -6032,10 +6032,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="C2">
-        <v>0.2712919611357874</v>
+        <v>1.410501914983034</v>
       </c>
     </row>
     <row r="3">
@@ -6486,10 +6486,10 @@
         </is>
       </c>
       <c r="C23">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D23">
-        <v>0.006134026491755945</v>
+        <v>0.006253658895711615</v>
       </c>
     </row>
     <row r="24">
@@ -6711,7 +6711,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>IGHG3</t>
+          <t>KRT10</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6720,46 +6720,46 @@
         </is>
       </c>
       <c r="C36">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D36">
-        <v>0.002033071723152557</v>
+        <v>0.002113686068996637</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>APOH</t>
+          <t>IGHG3</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>symbol</t>
+          <t>family</t>
         </is>
       </c>
       <c r="C37">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D37">
-        <v>0.001834766275260182</v>
+        <v>0.002033071723152557</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>KRT10</t>
+          <t>APOH</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>family</t>
+          <t>symbol</t>
         </is>
       </c>
       <c r="C38">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D38">
-        <v>0.001782338284746402</v>
+        <v>0.001834766275260182</v>
       </c>
     </row>
     <row r="39">
@@ -9933,7 +9933,7 @@
         </is>
       </c>
       <c r="C2">
-        <v>47.67588762314584</v>
+        <v>47.02304114647254</v>
       </c>
     </row>
     <row r="3">
@@ -9948,7 +9948,7 @@
         </is>
       </c>
       <c r="C3">
-        <v>32.94531359061347</v>
+        <v>32.55712075226026</v>
       </c>
     </row>
     <row r="4">
@@ -9963,7 +9963,7 @@
         </is>
       </c>
       <c r="C4">
-        <v>26.92237039484356</v>
+        <v>26.36469023306657</v>
       </c>
     </row>
     <row r="5">
@@ -9978,7 +9978,7 @@
         </is>
       </c>
       <c r="C5">
-        <v>44.22737005130872</v>
+        <v>43.53350247764178</v>
       </c>
     </row>
     <row r="6">
@@ -9993,7 +9993,7 @@
         </is>
       </c>
       <c r="C6">
-        <v>32.84756828876942</v>
+        <v>32.39487348948416</v>
       </c>
     </row>
     <row r="7">
@@ -10008,7 +10008,7 @@
         </is>
       </c>
       <c r="C7">
-        <v>33.77546156372504</v>
+        <v>33.31482870417345</v>
       </c>
     </row>
     <row r="8">
@@ -10023,7 +10023,7 @@
         </is>
       </c>
       <c r="C8">
-        <v>26.30610564617677</v>
+        <v>25.91978552525977</v>
       </c>
     </row>
     <row r="9">
@@ -10038,7 +10038,7 @@
         </is>
       </c>
       <c r="C9">
-        <v>30.12823711674234</v>
+        <v>29.72067622593642</v>
       </c>
     </row>
     <row r="10">
@@ -10053,7 +10053,7 @@
         </is>
       </c>
       <c r="C10">
-        <v>23.28056718797209</v>
+        <v>23.00692063974904</v>
       </c>
     </row>
     <row r="11">
@@ -10068,7 +10068,7 @@
         </is>
       </c>
       <c r="C11">
-        <v>23.85657703181791</v>
+        <v>23.33137910666068</v>
       </c>
     </row>
     <row r="12">
@@ -10083,7 +10083,7 @@
         </is>
       </c>
       <c r="C12">
-        <v>80.04730964967737</v>
+        <v>79.41277992510496</v>
       </c>
     </row>
     <row r="13">
@@ -10098,7 +10098,7 @@
         </is>
       </c>
       <c r="C13">
-        <v>47.56105652460237</v>
+        <v>47.01711075034413</v>
       </c>
     </row>
     <row r="14">
@@ -10113,7 +10113,7 @@
         </is>
       </c>
       <c r="C14">
-        <v>43.69280840733837</v>
+        <v>43.16364657622505</v>
       </c>
     </row>
     <row r="15">
@@ -10128,7 +10128,7 @@
         </is>
       </c>
       <c r="C15">
-        <v>21.18864330904015</v>
+        <v>20.78960794558883</v>
       </c>
     </row>
     <row r="16">
@@ -10143,7 +10143,7 @@
         </is>
       </c>
       <c r="C16">
-        <v>22.75198845249871</v>
+        <v>22.41970779267011</v>
       </c>
     </row>
     <row r="17">
@@ -10158,7 +10158,7 @@
         </is>
       </c>
       <c r="C17">
-        <v>42.15387739667176</v>
+        <v>41.51855872401673</v>
       </c>
     </row>
     <row r="18">
@@ -10173,7 +10173,7 @@
         </is>
       </c>
       <c r="C18">
-        <v>23.54008820945759</v>
+        <v>23.12442177215729</v>
       </c>
     </row>
     <row r="19">
@@ -10188,7 +10188,7 @@
         </is>
       </c>
       <c r="C19">
-        <v>29.38593188164029</v>
+        <v>28.8023231470601</v>
       </c>
     </row>
     <row r="20">
@@ -10203,7 +10203,7 @@
         </is>
       </c>
       <c r="C20">
-        <v>22.46195728590685</v>
+        <v>21.81614435383804</v>
       </c>
     </row>
     <row r="21">
@@ -10218,7 +10218,7 @@
         </is>
       </c>
       <c r="C21">
-        <v>20.35367056542408</v>
+        <v>19.76410868241904</v>
       </c>
     </row>
     <row r="22">
@@ -10233,7 +10233,7 @@
         </is>
       </c>
       <c r="C22">
-        <v>27.96902476406055</v>
+        <v>27.665080911571</v>
       </c>
     </row>
     <row r="23">
@@ -10248,7 +10248,7 @@
         </is>
       </c>
       <c r="C23">
-        <v>21.17139491633812</v>
+        <v>20.74119469340042</v>
       </c>
     </row>
     <row r="24">
@@ -10263,7 +10263,7 @@
         </is>
       </c>
       <c r="C24">
-        <v>23.87527495594478</v>
+        <v>23.44822584218077</v>
       </c>
     </row>
     <row r="25">
@@ -10278,7 +10278,7 @@
         </is>
       </c>
       <c r="C25">
-        <v>32.69182469649088</v>
+        <v>32.33712726566275</v>
       </c>
     </row>
     <row r="26">
@@ -10293,7 +10293,7 @@
         </is>
       </c>
       <c r="C26">
-        <v>30.93423891106747</v>
+        <v>30.61677370438202</v>
       </c>
     </row>
     <row r="27">
@@ -10308,7 +10308,7 @@
         </is>
       </c>
       <c r="C27">
-        <v>28.42310620817203</v>
+        <v>27.94241417164917</v>
       </c>
     </row>
     <row r="28">
@@ -10323,7 +10323,7 @@
         </is>
       </c>
       <c r="C28">
-        <v>16.63941848888081</v>
+        <v>16.1899190370299</v>
       </c>
     </row>
     <row r="29">
@@ -10338,7 +10338,7 @@
         </is>
       </c>
       <c r="C29">
-        <v>42.30503174963643</v>
+        <v>41.79544804452135</v>
       </c>
     </row>
     <row r="30">
@@ -10353,7 +10353,7 @@
         </is>
       </c>
       <c r="C30">
-        <v>34.37055072267925</v>
+        <v>33.75494497663782</v>
       </c>
     </row>
     <row r="31">
@@ -10368,7 +10368,7 @@
         </is>
       </c>
       <c r="C31">
-        <v>38.36347537032253</v>
+        <v>37.83783533605583</v>
       </c>
     </row>
     <row r="32">
@@ -10383,7 +10383,7 @@
         </is>
       </c>
       <c r="C32">
-        <v>47.64520736723398</v>
+        <v>47.08257216589515</v>
       </c>
     </row>
     <row r="33">
@@ -10398,7 +10398,7 @@
         </is>
       </c>
       <c r="C33">
-        <v>30.66402268078223</v>
+        <v>30.27778372464798</v>
       </c>
     </row>
     <row r="34">
@@ -10413,7 +10413,7 @@
         </is>
       </c>
       <c r="C34">
-        <v>39.74600589103538</v>
+        <v>39.24757045134573</v>
       </c>
     </row>
     <row r="35">
@@ -10428,7 +10428,7 @@
         </is>
       </c>
       <c r="C35">
-        <v>28.86995422984455</v>
+        <v>28.53269036525623</v>
       </c>
     </row>
     <row r="36">
@@ -10443,7 +10443,7 @@
         </is>
       </c>
       <c r="C36">
-        <v>28.14711412007461</v>
+        <v>27.86215322851367</v>
       </c>
     </row>
     <row r="37">
@@ -10458,7 +10458,7 @@
         </is>
       </c>
       <c r="C37">
-        <v>39.66854222119643</v>
+        <v>38.99885603345047</v>
       </c>
     </row>
     <row r="38">
@@ -10473,7 +10473,7 @@
         </is>
       </c>
       <c r="C38">
-        <v>45.34839915363387</v>
+        <v>44.82306792659711</v>
       </c>
     </row>
     <row r="39">
@@ -10488,7 +10488,7 @@
         </is>
       </c>
       <c r="C39">
-        <v>27.00680589104332</v>
+        <v>26.57507930736779</v>
       </c>
     </row>
     <row r="40">
@@ -10503,7 +10503,7 @@
         </is>
       </c>
       <c r="C40">
-        <v>41.67922369256501</v>
+        <v>41.15886138301373</v>
       </c>
     </row>
     <row r="41">
@@ -10518,7 +10518,7 @@
         </is>
       </c>
       <c r="C41">
-        <v>21.71493658086321</v>
+        <v>21.3813108471553</v>
       </c>
     </row>
     <row r="42">
@@ -10533,7 +10533,7 @@
         </is>
       </c>
       <c r="C42">
-        <v>48.19129352447257</v>
+        <v>47.22411699139989</v>
       </c>
     </row>
     <row r="43">
@@ -10548,7 +10548,7 @@
         </is>
       </c>
       <c r="C43">
-        <v>31.81801040014127</v>
+        <v>31.35766045589506</v>
       </c>
     </row>
     <row r="44">
@@ -10563,7 +10563,7 @@
         </is>
       </c>
       <c r="C44">
-        <v>41.90130733169551</v>
+        <v>41.42973355987387</v>
       </c>
     </row>
     <row r="45">
@@ -10578,7 +10578,7 @@
         </is>
       </c>
       <c r="C45">
-        <v>31.53510281837602</v>
+        <v>30.9875295545985</v>
       </c>
     </row>
     <row r="46">
@@ -10593,7 +10593,7 @@
         </is>
       </c>
       <c r="C46">
-        <v>38.16586452970394</v>
+        <v>37.59443858883385</v>
       </c>
     </row>
     <row r="47">
@@ -10608,7 +10608,7 @@
         </is>
       </c>
       <c r="C47">
-        <v>27.94183611072752</v>
+        <v>27.47456443444379</v>
       </c>
     </row>
     <row r="48">
@@ -10623,7 +10623,7 @@
         </is>
       </c>
       <c r="C48">
-        <v>36.60418227648745</v>
+        <v>36.06859609991601</v>
       </c>
     </row>
     <row r="49">
@@ -10638,7 +10638,7 @@
         </is>
       </c>
       <c r="C49">
-        <v>35.59251471492991</v>
+        <v>35.07818112870507</v>
       </c>
     </row>
     <row r="50">
@@ -10653,7 +10653,7 @@
         </is>
       </c>
       <c r="C50">
-        <v>39.43944411093926</v>
+        <v>38.82249670301957</v>
       </c>
     </row>
     <row r="51">
@@ -10668,7 +10668,7 @@
         </is>
       </c>
       <c r="C51">
-        <v>19.83335642665108</v>
+        <v>19.40669787966587</v>
       </c>
     </row>
     <row r="52">
@@ -10683,7 +10683,7 @@
         </is>
       </c>
       <c r="C52">
-        <v>30.26778016834878</v>
+        <v>29.74288286621121</v>
       </c>
     </row>
     <row r="53">
@@ -10698,7 +10698,7 @@
         </is>
       </c>
       <c r="C53">
-        <v>26.76418571869921</v>
+        <v>26.19707386979336</v>
       </c>
     </row>
     <row r="54">
@@ -10713,7 +10713,7 @@
         </is>
       </c>
       <c r="C54">
-        <v>21.70452816943379</v>
+        <v>21.14444414823692</v>
       </c>
     </row>
     <row r="55">
@@ -10728,7 +10728,7 @@
         </is>
       </c>
       <c r="C55">
-        <v>26.78763204874603</v>
+        <v>26.30759634947111</v>
       </c>
     </row>
     <row r="56">
@@ -10743,7 +10743,7 @@
         </is>
       </c>
       <c r="C56">
-        <v>14.61785164370152</v>
+        <v>14.30529212770564</v>
       </c>
     </row>
     <row r="57">
@@ -10758,7 +10758,7 @@
         </is>
       </c>
       <c r="C57">
-        <v>46.26017565198951</v>
+        <v>45.33570716849891</v>
       </c>
     </row>
     <row r="58">
@@ -10773,7 +10773,7 @@
         </is>
       </c>
       <c r="C58">
-        <v>33.30886079618666</v>
+        <v>32.74771956203917</v>
       </c>
     </row>
     <row r="59">
@@ -10788,7 +10788,7 @@
         </is>
       </c>
       <c r="C59">
-        <v>56.12512896531096</v>
+        <v>55.4344543452866</v>
       </c>
     </row>
     <row r="60">
@@ -10803,7 +10803,7 @@
         </is>
       </c>
       <c r="C60">
-        <v>44.93578198376525</v>
+        <v>44.4711413374326</v>
       </c>
     </row>
     <row r="61">
@@ -10818,7 +10818,7 @@
         </is>
       </c>
       <c r="C61">
-        <v>36.62097245644279</v>
+        <v>36.10698320190033</v>
       </c>
     </row>
     <row r="62">
@@ -10833,7 +10833,7 @@
         </is>
       </c>
       <c r="C62">
-        <v>29.93956069031647</v>
+        <v>29.53775686568815</v>
       </c>
     </row>
     <row r="63">
@@ -10848,7 +10848,7 @@
         </is>
       </c>
       <c r="C63">
-        <v>15.94567341877486</v>
+        <v>15.68028677811165</v>
       </c>
     </row>
     <row r="64">
@@ -10863,7 +10863,7 @@
         </is>
       </c>
       <c r="C64">
-        <v>35.80492528665793</v>
+        <v>35.36732170676791</v>
       </c>
     </row>
     <row r="65">
@@ -10878,7 +10878,7 @@
         </is>
       </c>
       <c r="C65">
-        <v>22.7417335321488</v>
+        <v>22.00027366056602</v>
       </c>
     </row>
     <row r="66">
@@ -10893,7 +10893,7 @@
         </is>
       </c>
       <c r="C66">
-        <v>16.8602152144968</v>
+        <v>16.46987812274428</v>
       </c>
     </row>
     <row r="67">
@@ -10908,7 +10908,7 @@
         </is>
       </c>
       <c r="C67">
-        <v>35.99984187396467</v>
+        <v>35.32377090866756</v>
       </c>
     </row>
     <row r="68">
@@ -10923,7 +10923,7 @@
         </is>
       </c>
       <c r="C68">
-        <v>16.69561257390728</v>
+        <v>16.25316576093141</v>
       </c>
     </row>
     <row r="69">
@@ -10938,7 +10938,7 @@
         </is>
       </c>
       <c r="C69">
-        <v>23.20450141981969</v>
+        <v>22.33322434816081</v>
       </c>
     </row>
     <row r="70">
@@ -10953,7 +10953,7 @@
         </is>
       </c>
       <c r="C70">
-        <v>20.57305290455586</v>
+        <v>20.02466439238577</v>
       </c>
     </row>
     <row r="71">
@@ -10968,7 +10968,7 @@
         </is>
       </c>
       <c r="C71">
-        <v>34.79292282301629</v>
+        <v>33.91084351027875</v>
       </c>
     </row>
     <row r="72">
@@ -10983,7 +10983,7 @@
         </is>
       </c>
       <c r="C72">
-        <v>34.06564329310944</v>
+        <v>33.21445435216213</v>
       </c>
     </row>
     <row r="73">
@@ -10998,7 +10998,7 @@
         </is>
       </c>
       <c r="C73">
-        <v>10.96343246605272</v>
+        <v>10.62154259844766</v>
       </c>
     </row>
     <row r="74">
@@ -11013,7 +11013,7 @@
         </is>
       </c>
       <c r="C74">
-        <v>7.969572023574983</v>
+        <v>7.782668652160243</v>
       </c>
     </row>
     <row r="75">
@@ -11028,7 +11028,7 @@
         </is>
       </c>
       <c r="C75">
-        <v>16.74537085623831</v>
+        <v>16.17444837136415</v>
       </c>
     </row>
     <row r="76">
@@ -11043,7 +11043,7 @@
         </is>
       </c>
       <c r="C76">
-        <v>29.87067839546477</v>
+        <v>29.10835215374552</v>
       </c>
     </row>
     <row r="77">
@@ -11058,7 +11058,7 @@
         </is>
       </c>
       <c r="C77">
-        <v>16.91498872609365</v>
+        <v>16.27938001938308</v>
       </c>
     </row>
     <row r="78">
@@ -11073,7 +11073,7 @@
         </is>
       </c>
       <c r="C78">
-        <v>39.54245235445715</v>
+        <v>38.62906150189742</v>
       </c>
     </row>
     <row r="79">
@@ -11088,7 +11088,7 @@
         </is>
       </c>
       <c r="C79">
-        <v>24.60595487784461</v>
+        <v>24.05635812904976</v>
       </c>
     </row>
     <row r="80">
@@ -11103,7 +11103,7 @@
         </is>
       </c>
       <c r="C80">
-        <v>28.91965199581156</v>
+        <v>28.25213139230239</v>
       </c>
     </row>
     <row r="81">
@@ -11118,7 +11118,7 @@
         </is>
       </c>
       <c r="C81">
-        <v>21.61977225324352</v>
+        <v>21.10609330728778</v>
       </c>
     </row>
     <row r="82">
@@ -11133,7 +11133,7 @@
         </is>
       </c>
       <c r="C82">
-        <v>30.38060629001883</v>
+        <v>29.40162936936815</v>
       </c>
     </row>
     <row r="83">
@@ -11148,7 +11148,7 @@
         </is>
       </c>
       <c r="C83">
-        <v>12.70941514144465</v>
+        <v>12.36875269109519</v>
       </c>
     </row>
     <row r="84">
@@ -11163,7 +11163,7 @@
         </is>
       </c>
       <c r="C84">
-        <v>41.06654871542835</v>
+        <v>40.13635924028212</v>
       </c>
     </row>
     <row r="85">
@@ -11178,7 +11178,7 @@
         </is>
       </c>
       <c r="C85">
-        <v>36.99648992657553</v>
+        <v>35.85289791285165</v>
       </c>
     </row>
     <row r="86">
@@ -11193,7 +11193,7 @@
         </is>
       </c>
       <c r="C86">
-        <v>24.45009777568204</v>
+        <v>23.67720609109429</v>
       </c>
     </row>
     <row r="87">
@@ -11208,7 +11208,7 @@
         </is>
       </c>
       <c r="C87">
-        <v>24.71441180559659</v>
+        <v>24.1043917514429</v>
       </c>
     </row>
     <row r="88">
@@ -11223,7 +11223,7 @@
         </is>
       </c>
       <c r="C88">
-        <v>52.97662653530515</v>
+        <v>51.87613995294066</v>
       </c>
     </row>
     <row r="89">
@@ -11238,7 +11238,7 @@
         </is>
       </c>
       <c r="C89">
-        <v>38.96394370949655</v>
+        <v>38.07796717189294</v>
       </c>
     </row>
     <row r="90">
@@ -11253,7 +11253,7 @@
         </is>
       </c>
       <c r="C90">
-        <v>23.84487039831377</v>
+        <v>23.0200033853911</v>
       </c>
     </row>
     <row r="91">
@@ -11268,7 +11268,7 @@
         </is>
       </c>
       <c r="C91">
-        <v>26.03918565573812</v>
+        <v>25.28632366281217</v>
       </c>
     </row>
     <row r="92">
@@ -11283,7 +11283,7 @@
         </is>
       </c>
       <c r="C92">
-        <v>25.36370339452061</v>
+        <v>24.84623514574021</v>
       </c>
     </row>
     <row r="93">
@@ -11298,7 +11298,7 @@
         </is>
       </c>
       <c r="C93">
-        <v>15.37613566725733</v>
+        <v>14.68360585458952</v>
       </c>
     </row>
     <row r="94">
@@ -11313,7 +11313,7 @@
         </is>
       </c>
       <c r="C94">
-        <v>29.66137073655472</v>
+        <v>28.99053523340854</v>
       </c>
     </row>
     <row r="95">
@@ -11328,7 +11328,7 @@
         </is>
       </c>
       <c r="C95">
-        <v>21.10797206848373</v>
+        <v>20.62496469476384</v>
       </c>
     </row>
     <row r="96">
@@ -11343,7 +11343,7 @@
         </is>
       </c>
       <c r="C96">
-        <v>12.31488381482708</v>
+        <v>11.81995629532636</v>
       </c>
     </row>
     <row r="97">
@@ -11358,7 +11358,7 @@
         </is>
       </c>
       <c r="C97">
-        <v>26.06550270766389</v>
+        <v>25.18378146704233</v>
       </c>
     </row>
     <row r="98">
@@ -11373,7 +11373,7 @@
         </is>
       </c>
       <c r="C98">
-        <v>21.86709376479077</v>
+        <v>21.2213137716085</v>
       </c>
     </row>
     <row r="99">
@@ -11388,7 +11388,7 @@
         </is>
       </c>
       <c r="C99">
-        <v>56.91174655003424</v>
+        <v>55.71645006919081</v>
       </c>
     </row>
     <row r="100">
@@ -11403,7 +11403,7 @@
         </is>
       </c>
       <c r="C100">
-        <v>19.4494897405777</v>
+        <v>18.61534360318008</v>
       </c>
     </row>
     <row r="101">
@@ -11418,7 +11418,7 @@
         </is>
       </c>
       <c r="C101">
-        <v>25.7404046871725</v>
+        <v>24.87606109496862</v>
       </c>
     </row>
     <row r="102">
@@ -11433,7 +11433,7 @@
         </is>
       </c>
       <c r="C102">
-        <v>39.20822070311088</v>
+        <v>38.50526962048674</v>
       </c>
     </row>
     <row r="103">
@@ -11448,7 +11448,7 @@
         </is>
       </c>
       <c r="C103">
-        <v>23.22997484491086</v>
+        <v>22.3454022062665</v>
       </c>
     </row>
     <row r="104">
@@ -11463,7 +11463,7 @@
         </is>
       </c>
       <c r="C104">
-        <v>21.00803406083094</v>
+        <v>20.41731302633366</v>
       </c>
     </row>
     <row r="105">
@@ -11478,7 +11478,7 @@
         </is>
       </c>
       <c r="C105">
-        <v>20.77715452642849</v>
+        <v>20.00415942702988</v>
       </c>
     </row>
     <row r="106">
@@ -11493,7 +11493,7 @@
         </is>
       </c>
       <c r="C106">
-        <v>39.97566362823648</v>
+        <v>39.0403313111988</v>
       </c>
     </row>
     <row r="107">
@@ -11508,7 +11508,7 @@
         </is>
       </c>
       <c r="C107">
-        <v>25.2190042862803</v>
+        <v>24.73678834546828</v>
       </c>
     </row>
     <row r="108">
@@ -11523,7 +11523,7 @@
         </is>
       </c>
       <c r="C108">
-        <v>29.09747088402708</v>
+        <v>28.19668867406861</v>
       </c>
     </row>
     <row r="109">
@@ -11538,7 +11538,7 @@
         </is>
       </c>
       <c r="C109">
-        <v>12.76292426989062</v>
+        <v>12.34855414156156</v>
       </c>
     </row>
     <row r="110">
@@ -11553,7 +11553,7 @@
         </is>
       </c>
       <c r="C110">
-        <v>27.88902870682065</v>
+        <v>27.2968076000766</v>
       </c>
     </row>
     <row r="111">
@@ -11568,7 +11568,7 @@
         </is>
       </c>
       <c r="C111">
-        <v>25.46757510230898</v>
+        <v>24.74929387641738</v>
       </c>
     </row>
     <row r="112">
@@ -11583,7 +11583,7 @@
         </is>
       </c>
       <c r="C112">
-        <v>11.80556463739358</v>
+        <v>11.32106377510243</v>
       </c>
     </row>
     <row r="113">
@@ -11598,7 +11598,7 @@
         </is>
       </c>
       <c r="C113">
-        <v>39.3487605731198</v>
+        <v>38.6779526640965</v>
       </c>
     </row>
     <row r="114">
@@ -11613,7 +11613,7 @@
         </is>
       </c>
       <c r="C114">
-        <v>18.15335844244948</v>
+        <v>17.46522941528066</v>
       </c>
     </row>
     <row r="115">
@@ -11628,7 +11628,7 @@
         </is>
       </c>
       <c r="C115">
-        <v>34.02997538438925</v>
+        <v>33.28622787292586</v>
       </c>
     </row>
     <row r="116">
@@ -11643,7 +11643,7 @@
         </is>
       </c>
       <c r="C116">
-        <v>32.71684271846188</v>
+        <v>32.14303518820611</v>
       </c>
     </row>
     <row r="117">
@@ -11658,7 +11658,7 @@
         </is>
       </c>
       <c r="C117">
-        <v>36.42309241970267</v>
+        <v>35.80329102007341</v>
       </c>
     </row>
     <row r="118">
@@ -11673,7 +11673,7 @@
         </is>
       </c>
       <c r="C118">
-        <v>7.030525483221525</v>
+        <v>6.757740060888698</v>
       </c>
     </row>
     <row r="119">
@@ -11688,7 +11688,7 @@
         </is>
       </c>
       <c r="C119">
-        <v>18.83582962865379</v>
+        <v>18.21229704246289</v>
       </c>
     </row>
     <row r="120">
@@ -11703,7 +11703,7 @@
         </is>
       </c>
       <c r="C120">
-        <v>20.84774351157882</v>
+        <v>20.37782248159677</v>
       </c>
     </row>
     <row r="121">
@@ -11718,7 +11718,7 @@
         </is>
       </c>
       <c r="C121">
-        <v>20.64031541564402</v>
+        <v>20.20620990733237</v>
       </c>
     </row>
     <row r="122">
@@ -11733,7 +11733,7 @@
         </is>
       </c>
       <c r="C122">
-        <v>47.02820160443556</v>
+        <v>46.07573446289673</v>
       </c>
     </row>
     <row r="123">
@@ -11748,7 +11748,7 @@
         </is>
       </c>
       <c r="C123">
-        <v>27.16603170315223</v>
+        <v>26.3548639993495</v>
       </c>
     </row>
     <row r="124">
@@ -11763,7 +11763,7 @@
         </is>
       </c>
       <c r="C124">
-        <v>32.2471799147256</v>
+        <v>31.57949128308851</v>
       </c>
     </row>
     <row r="125">
@@ -11778,7 +11778,7 @@
         </is>
       </c>
       <c r="C125">
-        <v>23.18245701507416</v>
+        <v>22.67509996788293</v>
       </c>
     </row>
     <row r="126">
@@ -11793,7 +11793,7 @@
         </is>
       </c>
       <c r="C126">
-        <v>21.29972454452716</v>
+        <v>20.54870208919165</v>
       </c>
     </row>
     <row r="127">
@@ -11808,7 +11808,7 @@
         </is>
       </c>
       <c r="C127">
-        <v>36.83350895420893</v>
+        <v>36.0808672410994</v>
       </c>
     </row>
     <row r="128">
@@ -11823,7 +11823,7 @@
         </is>
       </c>
       <c r="C128">
-        <v>16.40526740598066</v>
+        <v>15.67535986341749</v>
       </c>
     </row>
     <row r="129">
@@ -11838,7 +11838,7 @@
         </is>
       </c>
       <c r="C129">
-        <v>40.84166261694882</v>
+        <v>40.11378823216777</v>
       </c>
     </row>
     <row r="130">
@@ -11853,7 +11853,7 @@
         </is>
       </c>
       <c r="C130">
-        <v>30.97555630635593</v>
+        <v>30.44883651869334</v>
       </c>
     </row>
     <row r="131">
@@ -11868,7 +11868,7 @@
         </is>
       </c>
       <c r="C131">
-        <v>33.04784603373193</v>
+        <v>32.53221043689534</v>
       </c>
     </row>
     <row r="132">
@@ -11883,7 +11883,7 @@
         </is>
       </c>
       <c r="C132">
-        <v>49.3457184924102</v>
+        <v>48.65647028814254</v>
       </c>
     </row>
   </sheetData>

</xml_diff>